<commit_message>
Added id validation between CIR and pubchem
</commit_message>
<xml_diff>
--- a/data/cec_list.xlsx
+++ b/data/cec_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leighton\Documents\GitHub\STW\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF58FDD-6869-413C-9019-673195C78CB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E53AD0-1C7F-4B36-BEC6-1A60E74790C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16617" uniqueCount="4544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16617" uniqueCount="4546">
   <si>
     <t>Chemical Name</t>
   </si>
@@ -13676,7 +13676,13 @@
     <t>Tier 1 Screening</t>
   </si>
   <si>
-    <t>CAS</t>
+    <t>name</t>
+  </si>
+  <si>
+    <t>cas</t>
+  </si>
+  <si>
+    <t>label</t>
   </si>
 </sst>
 </file>
@@ -14013,13 +14019,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>4543</v>
       </c>
       <c r="B1" t="s">
-        <v>4543</v>
+        <v>4544</v>
       </c>
       <c r="C1" t="s">
-        <v>616</v>
+        <v>4545</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>